<commit_message>
Att Chamada 2B 28-08
</commit_message>
<xml_diff>
--- a/ds/turmas/2DES_B/frequencia-3-B.xlsx
+++ b/ds/turmas/2DES_B/frequencia-3-B.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sn1057928\Desktop\senai2026\ds\turmas\2DES_B\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sn1053361\Documents\senai2026\ds\turmas\2DES_B\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4CB09EA-076A-41C5-90C0-15FCD7A2B5AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D05274E-A7D9-4893-9AE2-C763D5828601}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1701" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1701" uniqueCount="46">
   <si>
     <t>Aluno</t>
   </si>
@@ -170,6 +170,9 @@
   </si>
   <si>
     <t>5P | F</t>
+  </si>
+  <si>
+    <t>5P|F</t>
   </si>
 </sst>
 </file>
@@ -719,7 +722,37 @@
     <cellStyle name="Título 4" xfId="5" builtinId="19" customBuiltin="1"/>
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="5">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -4073,7 +4106,7 @@
         <v>36</v>
       </c>
       <c r="BC15" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="CJ15" s="3"/>
       <c r="CK15" s="3"/>
@@ -7770,13 +7803,18 @@
   </sortState>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="D3:DE33">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="3" operator="equal">
       <formula>"F"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AZ3:AZ33">
+    <cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="F">
+      <formula>NOT(ISERROR(SEARCH("F",AZ3)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="BC5:BC33">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="F">
-      <formula>NOT(ISERROR(SEARCH("F",AZ3)))</formula>
+      <formula>NOT(ISERROR(SEARCH("F",BC5)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>